<commit_message>
docs: add formatted TEST_CASES.xlsx with manual test scripts and test execution results
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,46 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +72,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,268 +464,710 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Tên Test Case</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mã TC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Phân loại</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Các bước</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Dữ liệu kiểm thử</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Kết quả mong đợi</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>TC01</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Để trống Username và Password</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Hệ thống cảnh báo: Bạn chưa nhập tên đăng nhập</t>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang login
+2. Để trống cả 2 ô
+3. Click nút Đăng nhập</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>User: (Trống)
+Pass: (Trống)</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Hiển thị thông báo yêu cầu nhập tên đăng nhập/mật khẩu.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Hiển thị thông báo báo lỗi yêu cầu nhập.</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Theo log pytest</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>TC02</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Để trống Username, có nhập Password</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Hệ thống cảnh báo: Bạn chưa nhập tên đăng nhập</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Để trống Username, chỉ nhập Password</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang login
+2. Để trống ô Username
+3. Nhập Password hợp lệ
+4. Click nút Đăng nhập</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>User: (Trống)
+Pass: matkhau_batky</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hiển thị thông báo yêu cầu nhập tên đăng nhập.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Hiển thị thông báo báo lỗi yêu cầu nhập tên.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Theo log pytest</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>TC03</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Có nhập Username, để trống Password</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Hệ thống cảnh báo: Bạn chưa nhập mật khẩu</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Để trống Password, chỉ nhập Username</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang login
+2. Nhập Username hợp lệ
+3. Để trống ô Password
+4. Click nút Đăng nhập</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>User: masinhvien
+Pass: (Trống)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Hiển thị thông báo yêu cầu nhập mật khẩu.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Hiển thị thông báo báo lỗi yêu cầu mật khẩu.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Theo log pytest</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>TC04</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập bằng phím Enter</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Đăng nhập thành công, hệ thống chuyển hướng vào trang chủ</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang login
+2. Nhập Username và Password hợp lệ
+3. Nhấn phím Enter trên bàn phím thay vì click chuột</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>User: masinhvien
+Pass: matkhau</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Đăng nhập thành công, chuyển hướng vào trang chủ.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Test thất bại vì thông tin giả định không thể login thật.</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Cần thay thông tin thực tế vào code để pass.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>TC05</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Đăng nhập qua E-mail UTC (SSO)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Chuyển hướng sang cổng xác thực đăng nhập của Google</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Đăng nhập qua SSO (E-mail UTC)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang login
+2. Click nút 'Đăng nhập bằng e-mail UTC'</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Trình duyệt điều hướng sang trang xác thực của Google Workspace.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Đã chuyển hướng thành công sang trang SSO.</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Theo log pytest</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>TC06</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Chức năng Quên mật khẩu</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Chuyển sang màn hình khôi phục/đặt lại mật khẩu</t>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Kiểm tra chức năng Quên mật khẩu</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang login
+2. Click/Kiểm tra đường dẫn của 'Bạn quên mật khẩu đăng nhập?'</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Trỏ đến trang khôi phục mật khẩu (/Login/GetPass).</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Link thực tế đã trỏ đúng vào /Login/GetPass.</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Theo log pytest (sau khi fix HTML)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>TC07</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Kích hoạt cơ chế Mã bảo mật</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Màn hình tải lại, hiển thị hình ảnh CAPTCHA và ô nhập Mã bảo mật</t>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang login
+2. Cố tình nhập sai User/Pass 3 lần liên tiếp
+3. Kiểm tra trang web</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>User: user_sai
+Pass: pass_sai (3 lần)</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Hệ thống hiển thị thêm ô 'Mã bảo mật' và ảnh CAPTCHA.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Trang web đã tải và hiển thị CAPTCHA thành công.</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Theo log pytest (sau khi fix HTML)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>TC08</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Thay đổi (Làm mới) mã bảo mật</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Hình ảnh mã bảo mật (CAPTCHA) tải lại và hiển thị chuỗi ký tự mới</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Chức năng tải lại ảnh Mã bảo mật</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang có chứa CAPTCHA
+2. Click vào link 'đây' để yêu cầu đổi mã
+3. Kiểm tra src ảnh</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Đường dẫn (src) của ảnh CAPTCHA bị thay đổi để load ảnh mới.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Hệ thống đã tự động gán mã ngẫu nhiên để tải ảnh mới.</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Theo log pytest</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>TC09</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Để trống ô Mã bảo mật</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Hệ thống cảnh báo yêu cầu nhập mã bảo mật</t>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang có chứa CAPTCHA
+2. Nhập User và Pass hợp lệ
+3. Để trống ô 'Mã bảo mật'
+4. Click nút Đăng nhập</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>User: masinhvien
+Pass: matkhau
+CAPTCHA: (Trống)</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Hệ thống cảnh báo yêu cầu nhập mã bảo mật. Không cho đăng nhập.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Đã hiển thị cảnh báo thiếu mã bảo mật.</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Theo log pytest</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>TC10</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Nhập sai Mã bảo mật</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Hệ thống thông báo lỗi sai mã bảo mật. CAPTCHA tự động tải lại</t>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang có chứa CAPTCHA
+2. Nhập User/Pass hợp lệ
+3. Cố tình nhập sai mã CAPTCHA hiển thị
+4. Click Đăng nhập</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>User: masinhvien
+Pass: matkhau
+CAPTCHA: MA_SAI_123</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Hệ thống báo sai mã bảo mật và TỰ ĐỘNG tải lại ảnh CAPTCHA mới.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Có báo lỗi nhưng ảnh CAPTCHA không được tự động tải lại (src không thay đổi).</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Theo log pytest</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>TC11</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Nhập đúng Mã bảo mật, nhưng sai User/Pass</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Thông báo Tài khoản hoặc mật khẩu không đúng. CAPTCHA tải lại</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Nhập đúng Mã bảo mật, sai User/Pass</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang có chứa CAPTCHA
+2. Nhập sai User hoặc Pass
+3. Nhập chính xác mã CAPTCHA (giả định)
+4. Click Đăng nhập</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>User: sai
+Pass: sai
+CAPTCHA: MA_DUNG</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Báo lỗi 'Tài khoản hoặc mật khẩu không đúng'. TỰ ĐỘNG tải lại CAPTCHA.</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Đã báo lỗi sai tài khoản nhưng ảnh CAPTCHA không tự tải lại mã mới.</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Theo log pytest</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>TC12</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập thành công khi có Mã bảo mật</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Đăng nhập thành công, chuyển hướng vào trang chủ</t>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>1. Mở trang có chứa CAPTCHA
+2. Nhập đúng User, Pass và Mã bảo mật
+3. Click Đăng nhập</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>User: masinhvien
+Pass: matkhau
+CAPTCHA: MA_DUNG</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Đăng nhập thành công, hệ thống chuyển hướng vào trang chủ.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Test thất bại vì thông tin giả định không thể login thật.</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Cần thay thông tin thực tế vào code để pass.</t>
         </is>
       </c>
     </row>

</xml_diff>